<commit_message>
improvements in the format
</commit_message>
<xml_diff>
--- a/scripts/AgriStack_Data_Template.xlsx
+++ b/scripts/AgriStack_Data_Template.xlsx
@@ -401,15 +401,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:C72"/>
   <cols>
-    <col min="1" max="1" width="40.83203125" customWidth="1"/>
-    <col min="2" max="2" width="80.83203125" customWidth="1"/>
+    <col min="1" max="1" width="38.83203125" customWidth="1"/>
+    <col min="2" max="2" width="72.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>AgriStack Dashboard — Data Entry Template</v>
+        <v>AgriStack Dashboard — Data Entry Template  (v2)</v>
       </c>
     </row>
     <row r="2">
@@ -419,237 +420,611 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v/>
+        <v>Generated: 24 June 2026</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>PURPOSE</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>This file is the single source of truth for the AgriStack Dashboard.</v>
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Fill in all 4 data sheets accurately. The data will be imported into the dashboard automatically.</v>
+        <v>PURPOSE</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>HOW TO USE</v>
+        <v>This file is the SINGLE SOURCE OF TRUTH for the AgriStack dashboard.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Step 1: Fill in the USE_CASES sheet — one row per use case.</v>
+        <v>All 4 data sheets must be filled accurately before importing.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Step 2: Fill in the STATES sheet — one row per state/UT.</v>
+        <v>Once filled, run:  node scripts/excel-to-data.js</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Step 3: Fill in the MAPPER_APIS sheet — one row per API mapper.</v>
+        <v>Then restart the dashboard:  npm run dev</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Step 4: Fill in the CONFIG sheet — dashboard settings.</v>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Step 5: Save the file as AgriStack_Data_Template.xlsx (keep the name exactly as is).</v>
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Step 6: Run the import command: node scripts/excel-to-data.js</v>
+        <v>USE_CASES SHEET — COLUMN-BY-COLUMN GUIDE</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Step 7: Restart the dashboard: npm run dev</v>
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>Column</v>
+      </c>
+      <c r="B16" t="str">
+        <v>What to enter</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Example</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SHEET GUIDE</v>
+        <v>A  ID</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Serial number. Do not change existing IDs. Add new rows at bottom with next number.</v>
+      </c>
+      <c r="C17" t="str">
+        <v>1, 2, 3 ...</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>USE_CASES sheet</v>
+        <v>B  Use Case Name</v>
       </c>
       <c r="B18" t="str">
-        <v>All use cases with status, category, department, mapper, and states applied</v>
+        <v>Full official name of the use case / scheme</v>
+      </c>
+      <c r="C18" t="str">
+        <v>PM Kisan</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>STATES sheet</v>
+        <v>C  Status</v>
       </c>
       <c r="B19" t="str">
-        <v>State-wise MoU, DCS, FR flags and API integration counts</v>
+        <v>EXACT value from: Live | In Progress | Complete | On Hold | Pending</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Live</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>MAPPER_APIS sheet</v>
+        <v>D  Category</v>
       </c>
       <c r="B20" t="str">
-        <v>All mapper API IDs with descriptions and state completion counts</v>
+        <v>EXACT value from: Central | State | Multi | Private</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Central</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>CONFIG sheet</v>
+        <v>E  Department / Implementing Agency</v>
       </c>
       <c r="B21" t="str">
-        <v>Dashboard-level data like enrolled farmer count and last-updated date</v>
+        <v>The department or organisation implementing this use case</v>
+      </c>
+      <c r="C21" t="str">
+        <v>DoA  or  NABARD  or  Maharashtra</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v/>
+        <v>F  State / UT  (State category only)</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Fill ONLY if Category = State. Enter the ONE state name. Leave blank for Central/Multi/Private.</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Maharashtra</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>ALLOWED VALUES (do not use anything else — exact spelling matters)</v>
+        <v>G  States Implemented In  (Central / Multi only)</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Fill ONLY if Category = Central or Multi. Enter ALL states where this scheme is implemented, comma-separated.</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Uttar Pradesh, Maharashtra, Gujarat</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Status (USE_CASES):</v>
+        <v>H  Mapper API ID</v>
       </c>
       <c r="B24" t="str">
-        <v>Live | In Progress | Complete | On Hold | Pending</v>
+        <v>The mapper API code(s). Leave blank if no mapper is assigned.</v>
+      </c>
+      <c r="C24" t="str">
+        <v>i1001:o1004</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Category (USE_CASES):</v>
+        <v>I  Go-Live Date</v>
       </c>
       <c r="B25" t="str">
-        <v>Central | State | Multi | Private</v>
+        <v>For Live status use cases only. Month and year when it went live.</v>
+      </c>
+      <c r="C25" t="str">
+        <v>January 2025</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>MoU / DCS / FR (STATES):</v>
+        <v>J  Portal / URL</v>
       </c>
       <c r="B26" t="str">
-        <v>Yes | No</v>
+        <v>Official portal link if available. Leave blank if none.</v>
+      </c>
+      <c r="C26" t="str">
+        <v>https://pmkisan.gov.in</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Integration Status (STATES):</v>
+        <v>K  Scheme / Programme</v>
       </c>
       <c r="B27" t="str">
-        <v>Active | Partial | MoU Only | Not Live | Pending</v>
+        <v>The parent scheme or programme this use case falls under.</v>
+      </c>
+      <c r="C27" t="str">
+        <v>PM-KISAN  or  PMFBY</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v/>
+        <v>L  Remarks / Notes</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Any context, caveats, or important notes.</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Integration via PFMS gateway</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>IMPORTANT NOTES</v>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>— The "States Applied" column in USE_CASES is ONLY for Central / Multi category schemes.</v>
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>— For State category schemes, leave "States Applied" blank.</v>
+        <v>STATES SHEET — COLUMN-BY-COLUMN GUIDE</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>— Enter multiple states separated by commas. Example: Uttar Pradesh, Maharashtra, Gujarat</v>
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>— Do NOT delete existing rows. You may add new rows at the bottom.</v>
+        <v>Column</v>
+      </c>
+      <c r="B33" t="str">
+        <v>What to enter</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Example</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>— Do NOT change column headers.</v>
+        <v>A  State / UT Name</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Official state name as per GoI</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Uttar Pradesh</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>— This file was generated on: 24 June 2026</v>
+        <v>B  Region</v>
+      </c>
+      <c r="B35" t="str">
+        <v>North / South / East / West / North-East / Central / Island</v>
+      </c>
+      <c r="C35" t="str">
+        <v>North</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>C  MoU Signed</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Yes or No</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>D  DCS Done</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Yes or No  (District Collector / State Data Sharing)</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>E  FR Done</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Yes or No  (Farmer Registry completed)</v>
+      </c>
+      <c r="C38" t="str">
+        <v>No</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>F  Total Mapper APIs</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Total number of mapper API types applicable (usually 16 or 24)</v>
+      </c>
+      <c r="C39" t="str">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>G  APIs Integrated (Done)</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Count of mapper APIs actually integrated/live for this state</v>
+      </c>
+      <c r="C40" t="str">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>H  Integration Status</v>
+      </c>
+      <c r="B41" t="str">
+        <v>EXACT value: Active | Partial | MoU Only | Not Live | Pending</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>I  Enrolled Farmers</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Number of farmers enrolled from this state (if known). Leave blank if unknown.</v>
+      </c>
+      <c r="C42" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>J  Remarks</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Any notes about this state</v>
+      </c>
+      <c r="C43" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>MAPPER_APIS SHEET — COLUMN-BY-COLUMN GUIDE</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Column</v>
+      </c>
+      <c r="B48" t="str">
+        <v>What to enter</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Example</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>A  Mapper API ID</v>
+      </c>
+      <c r="B49" t="str">
+        <v>The exact API identifier</v>
+      </c>
+      <c r="C49" t="str">
+        <v>i1001:o1001</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>B  Description</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Plain-English description of what this API returns</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Farmer Data by Farmer ID</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>C  States Done (count)</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Number of states where this API is fully integrated/live</v>
+      </c>
+      <c r="C51" t="str">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>D  Remarks</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Any notes</v>
+      </c>
+      <c r="C52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>ALLOWED VALUES (copy-paste exactly — spelling matters)</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Status (USE_CASES col C):</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Live   |   In Progress   |   Complete   |   On Hold   |   Pending</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Category (USE_CASES col D):</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Central   |   State   |   Multi   |   Private</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>MoU / DCS / FR (STATES):</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Yes   |   No</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Integration Status (STATES):</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Active   |   Partial   |   MoU Only   |   Not Live   |   Pending</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Region (STATES):</v>
+      </c>
+      <c r="B61" t="str">
+        <v>North   |   South   |   East   |   West   |   North-East   |   Central   |   Island</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>IMPORTANT RULES</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━━</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>1. Column F (State/UT) is ONLY for Category=State use cases. ONE state name only.</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2. Column G (States Implemented In) is ONLY for Category=Central or Multi. List ALL states, comma-separated.</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>3. For Category=Private, columns F and G should both be left blank.</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>4. Do NOT delete existing rows. Add new ones at the bottom.</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>5. Do NOT rename column headers.</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>6. Save the file as AgriStack_Data_Template.xlsx (exact filename).</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>7. After filling, run:  node scripts/excel-to-data.js</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B35"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C72"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:L79"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
+    <col min="1" max="1" width="4.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
     <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="26.83203125" customWidth="1"/>
-    <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.83203125" customWidth="1"/>
+    <col min="7" max="7" width="55.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="32.83203125" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" customWidth="1"/>
+    <col min="12" max="12" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" xml:space="preserve">
       <c r="A1" t="str">
         <v>ID</v>
       </c>
       <c r="B1" t="str">
         <v>Use Case Name</v>
       </c>
-      <c r="C1" t="str">
-        <v>Status</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Category</v>
+      <c r="C1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Status
+(Live / In Progress / Complete / On Hold / Pending)</v>
+      </c>
+      <c r="D1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Category
+(Central / State / Multi / Private)</v>
       </c>
       <c r="E1" t="str">
-        <v>Department / State</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Mapper API ID</v>
-      </c>
-      <c r="G1" t="str">
-        <v>States Applied (Central/Multi only — comma-separated)</v>
-      </c>
-      <c r="H1" t="str">
+        <v>Department / Implementing Agency</v>
+      </c>
+      <c r="F1" t="str" xml:space="preserve">
+        <v xml:space="preserve">State / UT
+(Fill ONLY if Category = State — ONE state name)</v>
+      </c>
+      <c r="G1" t="str" xml:space="preserve">
+        <v xml:space="preserve">States Implemented In
+(Fill ONLY if Category = Central or Multi — comma-separated list)</v>
+      </c>
+      <c r="H1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Mapper API ID
+(leave blank if none)</v>
+      </c>
+      <c r="I1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Go-Live Date
+(month &amp; year, for Live status)</v>
+      </c>
+      <c r="J1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Portal / URL
+(official link, optional)</v>
+      </c>
+      <c r="K1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Scheme / Programme
+(parent scheme name)</v>
+      </c>
+      <c r="L1" t="str">
         <v>Remarks / Notes</v>
       </c>
     </row>
@@ -670,12 +1045,24 @@
         <v>DoA</v>
       </c>
       <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
         <v>i1:o2</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>PM-KISAN</v>
+      </c>
+      <c r="L2" t="str">
         <v/>
       </c>
     </row>
@@ -696,12 +1083,24 @@
         <v>DoA</v>
       </c>
       <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
         <v>i1004:o1007</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
         <v/>
       </c>
     </row>
@@ -722,12 +1121,24 @@
         <v>Horticulture</v>
       </c>
       <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
         <v>i1002:o1004</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v>MIDH</v>
+      </c>
+      <c r="L4" t="str">
         <v/>
       </c>
     </row>
@@ -748,12 +1159,24 @@
         <v>DoA</v>
       </c>
       <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
         <v>i6:o2</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
         <v/>
       </c>
     </row>
@@ -782,6 +1205,18 @@
       <c r="H6" t="str">
         <v/>
       </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -800,12 +1235,24 @@
         <v>DoA</v>
       </c>
       <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
         <v>i5:o6</v>
       </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
         <v/>
       </c>
     </row>
@@ -834,6 +1281,18 @@
       <c r="H8" t="str">
         <v/>
       </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -852,12 +1311,24 @@
         <v>NAFED</v>
       </c>
       <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
         <v>i1:o1 &amp; i5:o3</v>
       </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
-      <c r="H9" t="str">
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
         <v/>
       </c>
     </row>
@@ -886,6 +1357,18 @@
       <c r="H10" t="str">
         <v/>
       </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -912,6 +1395,18 @@
       <c r="H11" t="str">
         <v/>
       </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v>NABARD</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -938,6 +1433,18 @@
       <c r="H12" t="str">
         <v/>
       </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v>PMFBY</v>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -956,12 +1463,24 @@
         <v>DoA</v>
       </c>
       <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
         <v>i2:o14</v>
       </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
-      <c r="H13" t="str">
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v>SHC</v>
+      </c>
+      <c r="L13" t="str">
         <v/>
       </c>
     </row>
@@ -982,12 +1501,24 @@
         <v>Maharashtra</v>
       </c>
       <c r="F14" t="str">
-        <v/>
+        <v>Maharashtra</v>
       </c>
       <c r="G14" t="str">
         <v/>
       </c>
       <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
         <v/>
       </c>
     </row>
@@ -1008,12 +1539,24 @@
         <v>Maharashtra</v>
       </c>
       <c r="F15" t="str">
+        <v>Maharashtra</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
         <v>i4:o4 &amp; i4:o7</v>
       </c>
-      <c r="G15" t="str">
-        <v/>
-      </c>
-      <c r="H15" t="str">
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
         <v/>
       </c>
     </row>
@@ -1034,12 +1577,24 @@
         <v>Maharashtra</v>
       </c>
       <c r="F16" t="str">
+        <v>Maharashtra</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
         <v>i4:o4v1</v>
       </c>
-      <c r="G16" t="str">
-        <v/>
-      </c>
-      <c r="H16" t="str">
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v>JanSamarth</v>
+      </c>
+      <c r="L16" t="str">
         <v/>
       </c>
     </row>
@@ -1060,12 +1615,24 @@
         <v>Odisha</v>
       </c>
       <c r="F17" t="str">
+        <v>Odisha</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
         <v>i1:o1 &amp; i5:o3</v>
       </c>
-      <c r="G17" t="str">
-        <v/>
-      </c>
-      <c r="H17" t="str">
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v>MSP</v>
+      </c>
+      <c r="L17" t="str">
         <v/>
       </c>
     </row>
@@ -1086,12 +1653,24 @@
         <v>Maharashtra</v>
       </c>
       <c r="F18" t="str">
-        <v/>
+        <v>Maharashtra</v>
       </c>
       <c r="G18" t="str">
         <v/>
       </c>
       <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v>MSP</v>
+      </c>
+      <c r="L18" t="str">
         <v/>
       </c>
     </row>
@@ -1112,12 +1691,24 @@
         <v>Madhya Pradesh</v>
       </c>
       <c r="F19" t="str">
-        <v/>
+        <v>Madhya Pradesh</v>
       </c>
       <c r="G19" t="str">
         <v/>
       </c>
       <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v>MSP</v>
+      </c>
+      <c r="L19" t="str">
         <v/>
       </c>
     </row>
@@ -1138,12 +1729,24 @@
         <v>Maharashtra</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>Maharashtra</v>
       </c>
       <c r="G20" t="str">
         <v/>
       </c>
       <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
         <v/>
       </c>
     </row>
@@ -1164,12 +1767,24 @@
         <v>Uttar Pradesh</v>
       </c>
       <c r="F21" t="str">
+        <v>Uttar Pradesh</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
         <v>i12:o20</v>
       </c>
-      <c r="G21" t="str">
-        <v/>
-      </c>
-      <c r="H21" t="str">
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
         <v/>
       </c>
     </row>
@@ -1190,12 +1805,24 @@
         <v>Andhra Pradesh</v>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>Andhra Pradesh</v>
       </c>
       <c r="G22" t="str">
         <v/>
       </c>
       <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
         <v/>
       </c>
     </row>
@@ -1216,12 +1843,24 @@
         <v>Madhya Pradesh</v>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>Madhya Pradesh</v>
       </c>
       <c r="G23" t="str">
         <v/>
       </c>
       <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
+        <v/>
+      </c>
+      <c r="L23" t="str">
         <v/>
       </c>
     </row>
@@ -1242,12 +1881,24 @@
         <v>Chhattisgarh</v>
       </c>
       <c r="F24" t="str">
-        <v/>
+        <v>Chhattisgarh</v>
       </c>
       <c r="G24" t="str">
         <v/>
       </c>
       <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
+        <v>MSP</v>
+      </c>
+      <c r="L24" t="str">
         <v/>
       </c>
     </row>
@@ -1268,12 +1919,24 @@
         <v>Uttar Pradesh</v>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>Uttar Pradesh</v>
       </c>
       <c r="G25" t="str">
         <v/>
       </c>
       <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v>MSP</v>
+      </c>
+      <c r="L25" t="str">
         <v/>
       </c>
     </row>
@@ -1294,12 +1957,24 @@
         <v>Tamil Nadu</v>
       </c>
       <c r="F26" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
         <v>i1002:o1004</v>
       </c>
-      <c r="G26" t="str">
-        <v/>
-      </c>
-      <c r="H26" t="str">
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
         <v/>
       </c>
     </row>
@@ -1320,12 +1995,24 @@
         <v>Gujarat</v>
       </c>
       <c r="F27" t="str">
-        <v/>
+        <v>Gujarat</v>
       </c>
       <c r="G27" t="str">
         <v/>
       </c>
       <c r="H27" t="str">
+        <v/>
+      </c>
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
+        <v>MSP</v>
+      </c>
+      <c r="L27" t="str">
         <v/>
       </c>
     </row>
@@ -1346,12 +2033,24 @@
         <v>Uttar Pradesh</v>
       </c>
       <c r="F28" t="str">
-        <v/>
+        <v>Uttar Pradesh</v>
       </c>
       <c r="G28" t="str">
         <v/>
       </c>
       <c r="H28" t="str">
+        <v/>
+      </c>
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
+        <v/>
+      </c>
+      <c r="L28" t="str">
         <v/>
       </c>
     </row>
@@ -1372,12 +2071,24 @@
         <v>Maharashtra</v>
       </c>
       <c r="F29" t="str">
-        <v/>
+        <v>Maharashtra</v>
       </c>
       <c r="G29" t="str">
         <v/>
       </c>
       <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
+        <v>PoCRA</v>
+      </c>
+      <c r="L29" t="str">
         <v/>
       </c>
     </row>
@@ -1398,12 +2109,24 @@
         <v>Odisha</v>
       </c>
       <c r="F30" t="str">
-        <v/>
+        <v>Odisha</v>
       </c>
       <c r="G30" t="str">
         <v/>
       </c>
       <c r="H30" t="str">
+        <v/>
+      </c>
+      <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
+        <v/>
+      </c>
+      <c r="L30" t="str">
         <v/>
       </c>
     </row>
@@ -1424,12 +2147,24 @@
         <v>Gujarat</v>
       </c>
       <c r="F31" t="str">
-        <v/>
+        <v>Gujarat</v>
       </c>
       <c r="G31" t="str">
         <v/>
       </c>
       <c r="H31" t="str">
+        <v/>
+      </c>
+      <c r="I31" t="str">
+        <v/>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
+        <v/>
+      </c>
+      <c r="L31" t="str">
         <v/>
       </c>
     </row>
@@ -1450,12 +2185,24 @@
         <v>Tripura</v>
       </c>
       <c r="F32" t="str">
-        <v/>
+        <v>Tripura</v>
       </c>
       <c r="G32" t="str">
         <v/>
       </c>
       <c r="H32" t="str">
+        <v/>
+      </c>
+      <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
+        <v/>
+      </c>
+      <c r="L32" t="str">
         <v/>
       </c>
     </row>
@@ -1476,12 +2223,24 @@
         <v>Madhya Pradesh</v>
       </c>
       <c r="F33" t="str">
-        <v/>
+        <v>Madhya Pradesh</v>
       </c>
       <c r="G33" t="str">
         <v/>
       </c>
       <c r="H33" t="str">
+        <v/>
+      </c>
+      <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
+        <v/>
+      </c>
+      <c r="L33" t="str">
         <v/>
       </c>
     </row>
@@ -1502,12 +2261,24 @@
         <v>Uttar Pradesh</v>
       </c>
       <c r="F34" t="str">
-        <v/>
+        <v>Uttar Pradesh</v>
       </c>
       <c r="G34" t="str">
         <v/>
       </c>
       <c r="H34" t="str">
+        <v/>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
+        <v>PMFBY</v>
+      </c>
+      <c r="L34" t="str">
         <v/>
       </c>
     </row>
@@ -1536,6 +2307,18 @@
       <c r="H35" t="str">
         <v/>
       </c>
+      <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
+        <v>CFRP</v>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -1554,12 +2337,24 @@
         <v>Rajasthan</v>
       </c>
       <c r="F36" t="str">
-        <v/>
+        <v>Rajasthan</v>
       </c>
       <c r="G36" t="str">
         <v/>
       </c>
       <c r="H36" t="str">
+        <v/>
+      </c>
+      <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
+        <v>MSP</v>
+      </c>
+      <c r="L36" t="str">
         <v/>
       </c>
     </row>
@@ -1580,13 +2375,25 @@
         <v>Multi-State</v>
       </c>
       <c r="F37" t="str">
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
         <v>i4:o4v1</v>
       </c>
-      <c r="G37" t="str">
-        <v/>
-      </c>
-      <c r="H37" t="str">
-        <v/>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
+        <v>JanSamarth</v>
+      </c>
+      <c r="L37" t="str">
+        <v>Covers TG, AP, OD</v>
       </c>
     </row>
     <row r="38">
@@ -1614,6 +2421,18 @@
       <c r="H38" t="str">
         <v/>
       </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
+        <v/>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -1632,12 +2451,24 @@
         <v>Kerala</v>
       </c>
       <c r="F39" t="str">
-        <v/>
+        <v>Kerala</v>
       </c>
       <c r="G39" t="str">
         <v/>
       </c>
       <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
+        <v/>
+      </c>
+      <c r="L39" t="str">
         <v/>
       </c>
     </row>
@@ -1658,12 +2489,24 @@
         <v>Madhya Pradesh</v>
       </c>
       <c r="F40" t="str">
+        <v>Madhya Pradesh</v>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
         <v>i16:o21</v>
       </c>
-      <c r="G40" t="str">
-        <v/>
-      </c>
-      <c r="H40" t="str">
+      <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+      <c r="K40" t="str">
+        <v>EUDR</v>
+      </c>
+      <c r="L40" t="str">
         <v/>
       </c>
     </row>
@@ -1684,12 +2527,24 @@
         <v>Madhya Pradesh</v>
       </c>
       <c r="F41" t="str">
-        <v/>
+        <v>Madhya Pradesh</v>
       </c>
       <c r="G41" t="str">
         <v/>
       </c>
       <c r="H41" t="str">
+        <v/>
+      </c>
+      <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
+      <c r="K41" t="str">
+        <v/>
+      </c>
+      <c r="L41" t="str">
         <v/>
       </c>
     </row>
@@ -1710,12 +2565,24 @@
         <v>Fisheries</v>
       </c>
       <c r="F42" t="str">
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+      <c r="H42" t="str">
         <v>i4:o4</v>
       </c>
-      <c r="G42" t="str">
-        <v/>
-      </c>
-      <c r="H42" t="str">
+      <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
+        <v>NFDP</v>
+      </c>
+      <c r="L42" t="str">
         <v/>
       </c>
     </row>
@@ -1744,6 +2611,18 @@
       <c r="H43" t="str">
         <v/>
       </c>
+      <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
+        <v/>
+      </c>
+      <c r="L43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -1762,12 +2641,24 @@
         <v>Tamil Nadu</v>
       </c>
       <c r="F44" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+      <c r="H44" t="str">
         <v>i1002:o1004</v>
       </c>
-      <c r="G44" t="str">
-        <v/>
-      </c>
-      <c r="H44" t="str">
+      <c r="I44" t="str">
+        <v/>
+      </c>
+      <c r="J44" t="str">
+        <v/>
+      </c>
+      <c r="K44" t="str">
+        <v/>
+      </c>
+      <c r="L44" t="str">
         <v/>
       </c>
     </row>
@@ -1796,6 +2687,18 @@
       <c r="H45" t="str">
         <v/>
       </c>
+      <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
+      <c r="K45" t="str">
+        <v/>
+      </c>
+      <c r="L45" t="str">
+        <v>Covers MH, CG, MP</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -1814,12 +2717,24 @@
         <v>Maharashtra</v>
       </c>
       <c r="F46" t="str">
-        <v/>
+        <v>Maharashtra</v>
       </c>
       <c r="G46" t="str">
         <v/>
       </c>
       <c r="H46" t="str">
+        <v/>
+      </c>
+      <c r="I46" t="str">
+        <v/>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+      <c r="K46" t="str">
+        <v>CCI</v>
+      </c>
+      <c r="L46" t="str">
         <v/>
       </c>
     </row>
@@ -1840,12 +2755,24 @@
         <v>Multi-State</v>
       </c>
       <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
         <v>i1002:o1001 i15:o19 i1004:o1006V2</v>
       </c>
-      <c r="G47" t="str">
-        <v/>
-      </c>
-      <c r="H47" t="str">
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+      <c r="K47" t="str">
+        <v>ePACS</v>
+      </c>
+      <c r="L47" t="str">
         <v/>
       </c>
     </row>
@@ -1874,6 +2801,18 @@
       <c r="H48" t="str">
         <v/>
       </c>
+      <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
+      <c r="K48" t="str">
+        <v>PACS</v>
+      </c>
+      <c r="L48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -1900,6 +2839,18 @@
       <c r="H49" t="str">
         <v/>
       </c>
+      <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+      <c r="K49" t="str">
+        <v>AHD</v>
+      </c>
+      <c r="L49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -1926,6 +2877,18 @@
       <c r="H50" t="str">
         <v/>
       </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+      <c r="K50" t="str">
+        <v>PM ASHA</v>
+      </c>
+      <c r="L50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -1952,6 +2915,18 @@
       <c r="H51" t="str">
         <v/>
       </c>
+      <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+      <c r="K51" t="str">
+        <v/>
+      </c>
+      <c r="L51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -1970,12 +2945,24 @@
         <v>Uttar Pradesh</v>
       </c>
       <c r="F52" t="str">
-        <v/>
+        <v>Uttar Pradesh</v>
       </c>
       <c r="G52" t="str">
         <v/>
       </c>
       <c r="H52" t="str">
+        <v/>
+      </c>
+      <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+      <c r="K52" t="str">
+        <v>KCC</v>
+      </c>
+      <c r="L52" t="str">
         <v/>
       </c>
     </row>
@@ -2004,6 +2991,18 @@
       <c r="H53" t="str">
         <v/>
       </c>
+      <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+      <c r="K53" t="str">
+        <v>NABARD</v>
+      </c>
+      <c r="L53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -2030,6 +3029,18 @@
       <c r="H54" t="str">
         <v/>
       </c>
+      <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+      <c r="K54" t="str">
+        <v>CFRP</v>
+      </c>
+      <c r="L54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -2048,12 +3059,24 @@
         <v>Maharashtra</v>
       </c>
       <c r="F55" t="str">
-        <v/>
+        <v>Maharashtra</v>
       </c>
       <c r="G55" t="str">
         <v/>
       </c>
       <c r="H55" t="str">
+        <v/>
+      </c>
+      <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+      <c r="K55" t="str">
+        <v/>
+      </c>
+      <c r="L55" t="str">
         <v/>
       </c>
     </row>
@@ -2074,12 +3097,24 @@
         <v>Madhya Pradesh</v>
       </c>
       <c r="F56" t="str">
-        <v/>
+        <v>Madhya Pradesh</v>
       </c>
       <c r="G56" t="str">
         <v/>
       </c>
       <c r="H56" t="str">
+        <v/>
+      </c>
+      <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+      <c r="K56" t="str">
+        <v/>
+      </c>
+      <c r="L56" t="str">
         <v/>
       </c>
     </row>
@@ -2100,12 +3135,24 @@
         <v>Madhya Pradesh</v>
       </c>
       <c r="F57" t="str">
-        <v/>
+        <v>Madhya Pradesh</v>
       </c>
       <c r="G57" t="str">
         <v/>
       </c>
       <c r="H57" t="str">
+        <v/>
+      </c>
+      <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+      <c r="K57" t="str">
+        <v/>
+      </c>
+      <c r="L57" t="str">
         <v/>
       </c>
     </row>
@@ -2126,12 +3173,24 @@
         <v>Uttar Pradesh</v>
       </c>
       <c r="F58" t="str">
-        <v/>
+        <v>Uttar Pradesh</v>
       </c>
       <c r="G58" t="str">
         <v/>
       </c>
       <c r="H58" t="str">
+        <v/>
+      </c>
+      <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
+      <c r="K58" t="str">
+        <v/>
+      </c>
+      <c r="L58" t="str">
         <v/>
       </c>
     </row>
@@ -2160,6 +3219,18 @@
       <c r="H59" t="str">
         <v/>
       </c>
+      <c r="I59" t="str">
+        <v/>
+      </c>
+      <c r="J59" t="str">
+        <v/>
+      </c>
+      <c r="K59" t="str">
+        <v/>
+      </c>
+      <c r="L59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -2186,6 +3257,18 @@
       <c r="H60" t="str">
         <v/>
       </c>
+      <c r="I60" t="str">
+        <v/>
+      </c>
+      <c r="J60" t="str">
+        <v/>
+      </c>
+      <c r="K60" t="str">
+        <v/>
+      </c>
+      <c r="L60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -2204,12 +3287,24 @@
         <v>Uttar Pradesh</v>
       </c>
       <c r="F61" t="str">
-        <v/>
+        <v>Uttar Pradesh</v>
       </c>
       <c r="G61" t="str">
         <v/>
       </c>
       <c r="H61" t="str">
+        <v/>
+      </c>
+      <c r="I61" t="str">
+        <v/>
+      </c>
+      <c r="J61" t="str">
+        <v/>
+      </c>
+      <c r="K61" t="str">
+        <v/>
+      </c>
+      <c r="L61" t="str">
         <v/>
       </c>
     </row>
@@ -2238,6 +3333,18 @@
       <c r="H62" t="str">
         <v/>
       </c>
+      <c r="I62" t="str">
+        <v/>
+      </c>
+      <c r="J62" t="str">
+        <v/>
+      </c>
+      <c r="K62" t="str">
+        <v/>
+      </c>
+      <c r="L62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -2264,6 +3371,18 @@
       <c r="H63" t="str">
         <v/>
       </c>
+      <c r="I63" t="str">
+        <v/>
+      </c>
+      <c r="J63" t="str">
+        <v/>
+      </c>
+      <c r="K63" t="str">
+        <v/>
+      </c>
+      <c r="L63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -2290,6 +3409,18 @@
       <c r="H64" t="str">
         <v/>
       </c>
+      <c r="I64" t="str">
+        <v/>
+      </c>
+      <c r="J64" t="str">
+        <v/>
+      </c>
+      <c r="K64" t="str">
+        <v/>
+      </c>
+      <c r="L64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65">
@@ -2316,6 +3447,18 @@
       <c r="H65" t="str">
         <v/>
       </c>
+      <c r="I65" t="str">
+        <v/>
+      </c>
+      <c r="J65" t="str">
+        <v/>
+      </c>
+      <c r="K65" t="str">
+        <v/>
+      </c>
+      <c r="L65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66">
@@ -2342,6 +3485,18 @@
       <c r="H66" t="str">
         <v/>
       </c>
+      <c r="I66" t="str">
+        <v/>
+      </c>
+      <c r="J66" t="str">
+        <v/>
+      </c>
+      <c r="K66" t="str">
+        <v/>
+      </c>
+      <c r="L66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67">
@@ -2368,6 +3523,18 @@
       <c r="H67" t="str">
         <v/>
       </c>
+      <c r="I67" t="str">
+        <v/>
+      </c>
+      <c r="J67" t="str">
+        <v/>
+      </c>
+      <c r="K67" t="str">
+        <v/>
+      </c>
+      <c r="L67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68">
@@ -2394,6 +3561,18 @@
       <c r="H68" t="str">
         <v/>
       </c>
+      <c r="I68" t="str">
+        <v/>
+      </c>
+      <c r="J68" t="str">
+        <v/>
+      </c>
+      <c r="K68" t="str">
+        <v/>
+      </c>
+      <c r="L68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69">
@@ -2420,6 +3599,18 @@
       <c r="H69" t="str">
         <v/>
       </c>
+      <c r="I69" t="str">
+        <v/>
+      </c>
+      <c r="J69" t="str">
+        <v/>
+      </c>
+      <c r="K69" t="str">
+        <v/>
+      </c>
+      <c r="L69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70">
@@ -2446,6 +3637,18 @@
       <c r="H70" t="str">
         <v/>
       </c>
+      <c r="I70" t="str">
+        <v/>
+      </c>
+      <c r="J70" t="str">
+        <v/>
+      </c>
+      <c r="K70" t="str">
+        <v/>
+      </c>
+      <c r="L70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71">
@@ -2472,6 +3675,18 @@
       <c r="H71" t="str">
         <v/>
       </c>
+      <c r="I71" t="str">
+        <v/>
+      </c>
+      <c r="J71" t="str">
+        <v/>
+      </c>
+      <c r="K71" t="str">
+        <v/>
+      </c>
+      <c r="L71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72">
@@ -2498,6 +3713,18 @@
       <c r="H72" t="str">
         <v/>
       </c>
+      <c r="I72" t="str">
+        <v/>
+      </c>
+      <c r="J72" t="str">
+        <v/>
+      </c>
+      <c r="K72" t="str">
+        <v/>
+      </c>
+      <c r="L72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73">
@@ -2524,6 +3751,18 @@
       <c r="H73" t="str">
         <v/>
       </c>
+      <c r="I73" t="str">
+        <v/>
+      </c>
+      <c r="J73" t="str">
+        <v/>
+      </c>
+      <c r="K73" t="str">
+        <v/>
+      </c>
+      <c r="L73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74">
@@ -2550,6 +3789,18 @@
       <c r="H74" t="str">
         <v/>
       </c>
+      <c r="I74" t="str">
+        <v/>
+      </c>
+      <c r="J74" t="str">
+        <v/>
+      </c>
+      <c r="K74" t="str">
+        <v/>
+      </c>
+      <c r="L74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75">
@@ -2576,6 +3827,18 @@
       <c r="H75" t="str">
         <v/>
       </c>
+      <c r="I75" t="str">
+        <v/>
+      </c>
+      <c r="J75" t="str">
+        <v/>
+      </c>
+      <c r="K75" t="str">
+        <v/>
+      </c>
+      <c r="L75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76">
@@ -2594,12 +3857,24 @@
         <v>Bihar</v>
       </c>
       <c r="F76" t="str">
-        <v/>
+        <v>Bihar</v>
       </c>
       <c r="G76" t="str">
         <v/>
       </c>
       <c r="H76" t="str">
+        <v/>
+      </c>
+      <c r="I76" t="str">
+        <v/>
+      </c>
+      <c r="J76" t="str">
+        <v/>
+      </c>
+      <c r="K76" t="str">
+        <v/>
+      </c>
+      <c r="L76" t="str">
         <v/>
       </c>
     </row>
@@ -2620,12 +3895,24 @@
         <v>Maharashtra</v>
       </c>
       <c r="F77" t="str">
-        <v/>
+        <v>Maharashtra</v>
       </c>
       <c r="G77" t="str">
         <v/>
       </c>
       <c r="H77" t="str">
+        <v/>
+      </c>
+      <c r="I77" t="str">
+        <v/>
+      </c>
+      <c r="J77" t="str">
+        <v/>
+      </c>
+      <c r="K77" t="str">
+        <v/>
+      </c>
+      <c r="L77" t="str">
         <v/>
       </c>
     </row>
@@ -2654,6 +3941,18 @@
       <c r="H78" t="str">
         <v/>
       </c>
+      <c r="I78" t="str">
+        <v/>
+      </c>
+      <c r="J78" t="str">
+        <v/>
+      </c>
+      <c r="K78" t="str">
+        <v/>
+      </c>
+      <c r="L78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79">
@@ -2672,59 +3971,86 @@
         <v>Rajasthan</v>
       </c>
       <c r="F79" t="str">
-        <v/>
+        <v>Rajasthan</v>
       </c>
       <c r="G79" t="str">
         <v/>
       </c>
       <c r="H79" t="str">
+        <v/>
+      </c>
+      <c r="I79" t="str">
+        <v/>
+      </c>
+      <c r="J79" t="str">
+        <v/>
+      </c>
+      <c r="K79" t="str">
+        <v>MSP</v>
+      </c>
+      <c r="L79" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H79"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L79"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:J29"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="26.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" xml:space="preserve">
       <c r="A1" t="str">
         <v>State / UT Name</v>
       </c>
-      <c r="B1" t="str">
-        <v>MoU Signed (Yes/No)</v>
-      </c>
-      <c r="C1" t="str">
-        <v>DCS Done (Yes/No)</v>
-      </c>
-      <c r="D1" t="str">
-        <v>FR Done (Yes/No)</v>
-      </c>
-      <c r="E1" t="str">
+      <c r="B1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Region
+(North/South/East/West/North-East/Central/Island)</v>
+      </c>
+      <c r="C1" t="str" xml:space="preserve">
+        <v xml:space="preserve">MoU Signed
+(Yes/No)</v>
+      </c>
+      <c r="D1" t="str" xml:space="preserve">
+        <v xml:space="preserve">DCS Done
+(Yes/No)</v>
+      </c>
+      <c r="E1" t="str" xml:space="preserve">
+        <v xml:space="preserve">FR Done
+(Yes/No)</v>
+      </c>
+      <c r="F1" t="str">
         <v>Total Mapper APIs</v>
       </c>
-      <c r="F1" t="str">
-        <v>APIs Integrated (Done count)</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Integration Status</v>
-      </c>
-      <c r="H1" t="str">
+      <c r="G1" t="str" xml:space="preserve">
+        <v xml:space="preserve">APIs Integrated
+(Done count)</v>
+      </c>
+      <c r="H1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Integration Status
+(Active/Partial/MoU Only/Not Live/Pending)</v>
+      </c>
+      <c r="I1" t="str" xml:space="preserve">
+        <v xml:space="preserve">Enrolled Farmers
+(number, if known)</v>
+      </c>
+      <c r="J1" t="str">
         <v>Remarks</v>
       </c>
     </row>
@@ -2733,7 +4059,7 @@
         <v>Gujarat</v>
       </c>
       <c r="B2" t="str">
-        <v>Yes</v>
+        <v>West</v>
       </c>
       <c r="C2" t="str">
         <v>Yes</v>
@@ -2741,16 +4067,22 @@
       <c r="D2" t="str">
         <v>Yes</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F2">
         <v>24</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>20</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Active</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v/>
       </c>
     </row>
@@ -2759,7 +4091,7 @@
         <v>Uttar Pradesh</v>
       </c>
       <c r="B3" t="str">
-        <v>Yes</v>
+        <v>North</v>
       </c>
       <c r="C3" t="str">
         <v>Yes</v>
@@ -2767,16 +4099,22 @@
       <c r="D3" t="str">
         <v>Yes</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F3">
         <v>24</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>22</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>Active</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v/>
       </c>
     </row>
@@ -2785,7 +4123,7 @@
         <v>Maharashtra</v>
       </c>
       <c r="B4" t="str">
-        <v>Yes</v>
+        <v>West</v>
       </c>
       <c r="C4" t="str">
         <v>Yes</v>
@@ -2793,16 +4131,22 @@
       <c r="D4" t="str">
         <v>Yes</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F4">
         <v>24</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>18</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Active</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v/>
       </c>
     </row>
@@ -2811,7 +4155,7 @@
         <v>Madhya Pradesh</v>
       </c>
       <c r="B5" t="str">
-        <v>Yes</v>
+        <v>Central</v>
       </c>
       <c r="C5" t="str">
         <v>Yes</v>
@@ -2819,16 +4163,22 @@
       <c r="D5" t="str">
         <v>Yes</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F5">
         <v>24</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>16</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>Active</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v/>
       </c>
     </row>
@@ -2837,7 +4187,7 @@
         <v>Odisha</v>
       </c>
       <c r="B6" t="str">
-        <v>Yes</v>
+        <v>East</v>
       </c>
       <c r="C6" t="str">
         <v>Yes</v>
@@ -2845,16 +4195,22 @@
       <c r="D6" t="str">
         <v>Yes</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F6">
         <v>24</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>17</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>Active</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
         <v/>
       </c>
     </row>
@@ -2863,7 +4219,7 @@
         <v>Andhra Pradesh</v>
       </c>
       <c r="B7" t="str">
-        <v>Yes</v>
+        <v>South</v>
       </c>
       <c r="C7" t="str">
         <v>Yes</v>
@@ -2871,16 +4227,22 @@
       <c r="D7" t="str">
         <v>Yes</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F7">
         <v>24</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>14</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>Active</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
         <v/>
       </c>
     </row>
@@ -2889,7 +4251,7 @@
         <v>Chhattisgarh</v>
       </c>
       <c r="B8" t="str">
-        <v>Yes</v>
+        <v>Central</v>
       </c>
       <c r="C8" t="str">
         <v>Yes</v>
@@ -2897,16 +4259,22 @@
       <c r="D8" t="str">
         <v>Yes</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F8">
         <v>24</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>16</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>Active</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
         <v/>
       </c>
     </row>
@@ -2915,7 +4283,7 @@
         <v>Tamil Nadu</v>
       </c>
       <c r="B9" t="str">
-        <v>Yes</v>
+        <v>South</v>
       </c>
       <c r="C9" t="str">
         <v>Yes</v>
@@ -2923,16 +4291,22 @@
       <c r="D9" t="str">
         <v>Yes</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F9">
         <v>24</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>14</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>Active</v>
       </c>
-      <c r="H9" t="str">
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
         <v/>
       </c>
     </row>
@@ -2941,7 +4315,7 @@
         <v>Rajasthan</v>
       </c>
       <c r="B10" t="str">
-        <v>Yes</v>
+        <v>North</v>
       </c>
       <c r="C10" t="str">
         <v>Yes</v>
@@ -2949,16 +4323,22 @@
       <c r="D10" t="str">
         <v>Yes</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F10">
         <v>24</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>13</v>
       </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>Active</v>
       </c>
-      <c r="H10" t="str">
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
         <v/>
       </c>
     </row>
@@ -2967,7 +4347,7 @@
         <v>Assam</v>
       </c>
       <c r="B11" t="str">
-        <v>Yes</v>
+        <v>North-East</v>
       </c>
       <c r="C11" t="str">
         <v>Yes</v>
@@ -2975,16 +4355,22 @@
       <c r="D11" t="str">
         <v>Yes</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F11">
         <v>24</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <v>14</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>Active</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
         <v/>
       </c>
     </row>
@@ -2993,7 +4379,7 @@
         <v>Telangana</v>
       </c>
       <c r="B12" t="str">
-        <v>Yes</v>
+        <v>South</v>
       </c>
       <c r="C12" t="str">
         <v>Yes</v>
@@ -3001,16 +4387,22 @@
       <c r="D12" t="str">
         <v>Yes</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F12">
         <v>24</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>12</v>
       </c>
-      <c r="G12" t="str">
+      <c r="H12" t="str">
         <v>Active</v>
       </c>
-      <c r="H12" t="str">
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
         <v/>
       </c>
     </row>
@@ -3019,7 +4411,7 @@
         <v>Punjab</v>
       </c>
       <c r="B13" t="str">
-        <v>Yes</v>
+        <v>North</v>
       </c>
       <c r="C13" t="str">
         <v>Yes</v>
@@ -3027,16 +4419,22 @@
       <c r="D13" t="str">
         <v>Yes</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F13">
         <v>24</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <v>11</v>
       </c>
-      <c r="G13" t="str">
+      <c r="H13" t="str">
         <v>Active</v>
       </c>
-      <c r="H13" t="str">
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
         <v/>
       </c>
     </row>
@@ -3045,7 +4443,7 @@
         <v>Bihar</v>
       </c>
       <c r="B14" t="str">
-        <v>Yes</v>
+        <v>East</v>
       </c>
       <c r="C14" t="str">
         <v>Yes</v>
@@ -3053,16 +4451,22 @@
       <c r="D14" t="str">
         <v>Yes</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F14">
         <v>24</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>9</v>
       </c>
-      <c r="G14" t="str">
+      <c r="H14" t="str">
         <v>Active</v>
       </c>
-      <c r="H14" t="str">
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
         <v/>
       </c>
     </row>
@@ -3071,7 +4475,7 @@
         <v>Kerala</v>
       </c>
       <c r="B15" t="str">
-        <v>Yes</v>
+        <v>South</v>
       </c>
       <c r="C15" t="str">
         <v>Yes</v>
@@ -3079,16 +4483,22 @@
       <c r="D15" t="str">
         <v>Yes</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F15">
         <v>24</v>
       </c>
-      <c r="F15">
+      <c r="G15">
         <v>8</v>
       </c>
-      <c r="G15" t="str">
+      <c r="H15" t="str">
         <v>Active</v>
       </c>
-      <c r="H15" t="str">
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
         <v/>
       </c>
     </row>
@@ -3097,7 +4507,7 @@
         <v>Karnataka</v>
       </c>
       <c r="B16" t="str">
-        <v>Yes</v>
+        <v>South</v>
       </c>
       <c r="C16" t="str">
         <v>Yes</v>
@@ -3105,16 +4515,22 @@
       <c r="D16" t="str">
         <v>Yes</v>
       </c>
-      <c r="E16">
+      <c r="E16" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F16">
         <v>24</v>
       </c>
-      <c r="F16">
+      <c r="G16">
         <v>6</v>
       </c>
-      <c r="G16" t="str">
+      <c r="H16" t="str">
         <v>Partial</v>
       </c>
-      <c r="H16" t="str">
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
         <v/>
       </c>
     </row>
@@ -3123,7 +4539,7 @@
         <v>Himachal Pradesh</v>
       </c>
       <c r="B17" t="str">
-        <v>Yes</v>
+        <v>North</v>
       </c>
       <c r="C17" t="str">
         <v>Yes</v>
@@ -3131,16 +4547,22 @@
       <c r="D17" t="str">
         <v>Yes</v>
       </c>
-      <c r="E17">
+      <c r="E17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F17">
         <v>24</v>
       </c>
-      <c r="F17">
+      <c r="G17">
         <v>6</v>
       </c>
-      <c r="G17" t="str">
+      <c r="H17" t="str">
         <v>Partial</v>
       </c>
-      <c r="H17" t="str">
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
         <v/>
       </c>
     </row>
@@ -3149,7 +4571,7 @@
         <v>Haryana</v>
       </c>
       <c r="B18" t="str">
-        <v>Yes</v>
+        <v>North</v>
       </c>
       <c r="C18" t="str">
         <v>Yes</v>
@@ -3157,16 +4579,22 @@
       <c r="D18" t="str">
         <v>Yes</v>
       </c>
-      <c r="E18">
+      <c r="E18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F18">
         <v>24</v>
       </c>
-      <c r="F18">
+      <c r="G18">
         <v>5</v>
       </c>
-      <c r="G18" t="str">
+      <c r="H18" t="str">
         <v>Partial</v>
       </c>
-      <c r="H18" t="str">
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
         <v/>
       </c>
     </row>
@@ -3175,24 +4603,30 @@
         <v>Tripura</v>
       </c>
       <c r="B19" t="str">
-        <v>Yes</v>
+        <v>North-East</v>
       </c>
       <c r="C19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="D19" t="str">
         <v>No</v>
       </c>
-      <c r="D19" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="E19">
+      <c r="E19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F19">
         <v>24</v>
       </c>
-      <c r="F19">
+      <c r="G19">
         <v>5</v>
       </c>
-      <c r="G19" t="str">
+      <c r="H19" t="str">
         <v>Partial</v>
       </c>
-      <c r="H19" t="str">
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
         <v/>
       </c>
     </row>
@@ -3201,7 +4635,7 @@
         <v>Uttarakhand</v>
       </c>
       <c r="B20" t="str">
-        <v>Yes</v>
+        <v>North</v>
       </c>
       <c r="C20" t="str">
         <v>Yes</v>
@@ -3209,16 +4643,22 @@
       <c r="D20" t="str">
         <v>Yes</v>
       </c>
-      <c r="E20">
+      <c r="E20" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="F20">
         <v>24</v>
       </c>
-      <c r="F20">
+      <c r="G20">
         <v>3</v>
       </c>
-      <c r="G20" t="str">
+      <c r="H20" t="str">
         <v>Partial</v>
       </c>
-      <c r="H20" t="str">
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
         <v/>
       </c>
     </row>
@@ -3227,24 +4667,30 @@
         <v>Jharkhand</v>
       </c>
       <c r="B21" t="str">
-        <v>Yes</v>
+        <v>East</v>
       </c>
       <c r="C21" t="str">
         <v>Yes</v>
       </c>
       <c r="D21" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E21" t="str">
         <v>No</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <v>24</v>
       </c>
-      <c r="F21">
+      <c r="G21">
         <v>1</v>
       </c>
-      <c r="G21" t="str">
+      <c r="H21" t="str">
         <v>Not Live</v>
       </c>
-      <c r="H21" t="str">
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
         <v/>
       </c>
     </row>
@@ -3253,24 +4699,30 @@
         <v>Manipur</v>
       </c>
       <c r="B22" t="str">
-        <v>Yes</v>
+        <v>North-East</v>
       </c>
       <c r="C22" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="D22" t="str">
         <v>No</v>
       </c>
-      <c r="E22">
+      <c r="E22" t="str">
+        <v>No</v>
+      </c>
+      <c r="F22">
         <v>24</v>
       </c>
-      <c r="F22">
+      <c r="G22">
         <v>4</v>
       </c>
-      <c r="G22" t="str">
+      <c r="H22" t="str">
         <v>Partial</v>
       </c>
-      <c r="H22" t="str">
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
         <v/>
       </c>
     </row>
@@ -3279,24 +4731,30 @@
         <v>Jammu &amp; Kashmir</v>
       </c>
       <c r="B23" t="str">
-        <v>Yes</v>
+        <v>North</v>
       </c>
       <c r="C23" t="str">
         <v>Yes</v>
       </c>
       <c r="D23" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E23" t="str">
         <v>No</v>
       </c>
-      <c r="E23">
+      <c r="F23">
         <v>24</v>
       </c>
-      <c r="F23">
+      <c r="G23">
         <v>0</v>
       </c>
-      <c r="G23" t="str">
+      <c r="H23" t="str">
         <v>MoU Only</v>
       </c>
-      <c r="H23" t="str">
+      <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
         <v/>
       </c>
     </row>
@@ -3305,24 +4763,30 @@
         <v>Puducherry</v>
       </c>
       <c r="B24" t="str">
-        <v>Yes</v>
+        <v>South</v>
       </c>
       <c r="C24" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="D24" t="str">
         <v>No</v>
       </c>
-      <c r="E24">
+      <c r="E24" t="str">
+        <v>No</v>
+      </c>
+      <c r="F24">
         <v>24</v>
       </c>
-      <c r="F24">
+      <c r="G24">
         <v>0</v>
       </c>
-      <c r="G24" t="str">
+      <c r="H24" t="str">
         <v>MoU Only</v>
       </c>
-      <c r="H24" t="str">
+      <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
         <v/>
       </c>
     </row>
@@ -3331,24 +4795,30 @@
         <v>Goa</v>
       </c>
       <c r="B25" t="str">
+        <v>West</v>
+      </c>
+      <c r="C25" t="str">
         <v>No</v>
       </c>
-      <c r="C25" t="str">
-        <v>Yes</v>
-      </c>
       <c r="D25" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E25" t="str">
         <v>No</v>
       </c>
-      <c r="E25">
+      <c r="F25">
         <v>24</v>
       </c>
-      <c r="F25">
+      <c r="G25">
         <v>0</v>
       </c>
-      <c r="G25" t="str">
+      <c r="H25" t="str">
         <v>MoU Only</v>
       </c>
-      <c r="H25" t="str">
+      <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
         <v/>
       </c>
     </row>
@@ -3357,24 +4827,30 @@
         <v>Mizoram</v>
       </c>
       <c r="B26" t="str">
-        <v>Yes</v>
+        <v>North-East</v>
       </c>
       <c r="C26" t="str">
         <v>Yes</v>
       </c>
       <c r="D26" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="E26" t="str">
         <v>No</v>
       </c>
-      <c r="E26">
+      <c r="F26">
         <v>24</v>
       </c>
-      <c r="F26">
+      <c r="G26">
         <v>0</v>
       </c>
-      <c r="G26" t="str">
+      <c r="H26" t="str">
         <v>MoU Only</v>
       </c>
-      <c r="H26" t="str">
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
         <v/>
       </c>
     </row>
@@ -3383,24 +4859,30 @@
         <v>Arunachal Pradesh</v>
       </c>
       <c r="B27" t="str">
-        <v>Yes</v>
+        <v>North-East</v>
       </c>
       <c r="C27" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="D27" t="str">
         <v>No</v>
       </c>
-      <c r="E27">
+      <c r="E27" t="str">
+        <v>No</v>
+      </c>
+      <c r="F27">
         <v>24</v>
       </c>
-      <c r="F27">
+      <c r="G27">
         <v>0</v>
       </c>
-      <c r="G27" t="str">
+      <c r="H27" t="str">
         <v>Pending</v>
       </c>
-      <c r="H27" t="str">
+      <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
         <v/>
       </c>
     </row>
@@ -3409,7 +4891,7 @@
         <v>Meghalaya</v>
       </c>
       <c r="B28" t="str">
-        <v>No</v>
+        <v>North-East</v>
       </c>
       <c r="C28" t="str">
         <v>No</v>
@@ -3417,16 +4899,22 @@
       <c r="D28" t="str">
         <v>No</v>
       </c>
-      <c r="E28">
+      <c r="E28" t="str">
+        <v>No</v>
+      </c>
+      <c r="F28">
         <v>24</v>
       </c>
-      <c r="F28">
+      <c r="G28">
         <v>0</v>
       </c>
-      <c r="G28" t="str">
+      <c r="H28" t="str">
         <v>Pending</v>
       </c>
-      <c r="H28" t="str">
+      <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
         <v/>
       </c>
     </row>
@@ -3435,7 +4923,7 @@
         <v>West Bengal</v>
       </c>
       <c r="B29" t="str">
-        <v>No</v>
+        <v>East</v>
       </c>
       <c r="C29" t="str">
         <v>No</v>
@@ -3443,22 +4931,28 @@
       <c r="D29" t="str">
         <v>No</v>
       </c>
-      <c r="E29">
+      <c r="E29" t="str">
+        <v>No</v>
+      </c>
+      <c r="F29">
         <v>24</v>
       </c>
-      <c r="F29">
+      <c r="G29">
         <v>0</v>
       </c>
-      <c r="G29" t="str">
+      <c r="H29" t="str">
         <v>Pending</v>
       </c>
-      <c r="H29" t="str">
+      <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3469,19 +4963,20 @@
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
-    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
     <col min="4" max="4" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" xml:space="preserve">
       <c r="A1" t="str">
         <v>Mapper API ID</v>
       </c>
       <c r="B1" t="str">
         <v>Description (what data this API provides)</v>
       </c>
-      <c r="C1" t="str">
-        <v>Total States Active (done count)</v>
+      <c r="C1" t="str" xml:space="preserve">
+        <v xml:space="preserve">States Done
+(count of states with this API integrated)</v>
       </c>
       <c r="D1" t="str">
         <v>Remarks</v>
@@ -3720,7 +5215,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C15"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="55.83203125" customWidth="1"/>
@@ -3735,7 +5230,7 @@
         <v>Value</v>
       </c>
       <c r="C1" t="str">
-        <v>Notes</v>
+        <v>Notes / Instructions</v>
       </c>
     </row>
     <row r="2">
@@ -3746,7 +5241,7 @@
         <v>99875423</v>
       </c>
       <c r="C2" t="str">
-        <v>Total farmer IDs enrolled on AgriStack. Update with latest figure.</v>
+        <v>Total farmer IDs enrolled on AgriStack. Verify and update.</v>
       </c>
     </row>
     <row r="3">
@@ -3757,7 +5252,7 @@
         <v>23 June 2026</v>
       </c>
       <c r="C3" t="str">
-        <v>Date when the enrolled farmer count was last verified.</v>
+        <v>Date when the enrolled farmer count was last checked. Format: DD Month YYYY</v>
       </c>
     </row>
     <row r="4">
@@ -3768,7 +5263,7 @@
         <v/>
       </c>
       <c r="C4" t="str">
-        <v>Date the Excel file was last filled/verified by team (e.g. 24 June 2026).</v>
+        <v>Date this Excel was last verified by team. Format: DD Month YYYY (e.g. 24 June 2026)</v>
       </c>
     </row>
     <row r="5">
@@ -3784,51 +5279,117 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Total Mapper APIs</v>
+        <v>Total Mapper API Types</v>
       </c>
       <c r="B6" t="str">
         <v>16</v>
       </c>
       <c r="C6" t="str">
-        <v>Total number of mapper API types tracked.</v>
+        <v>Total number of distinct mapper API types tracked.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Dashboard Subtitle</v>
+        <v>Total Use Cases</v>
       </c>
       <c r="B7" t="str">
-        <v>Digital Agriculture Mission — Use Case Command Centre</v>
+        <v>78</v>
       </c>
       <c r="C7" t="str">
-        <v>Appears in the hero banner.</v>
+        <v>Update if use cases are added or removed.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Ministry Name</v>
+        <v>Dashboard Title</v>
       </c>
       <c r="B8" t="str">
-        <v>Ministry of Agriculture &amp; Farmers Welfare, Government of India</v>
+        <v>AgriStack Use Case Command Centre</v>
       </c>
       <c r="C8" t="str">
-        <v/>
+        <v>Appears in the browser tab.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Dashboard Subtitle</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Digital Agriculture Mission — Use Case Command Centre</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Appears in the hero banner.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Ministry Name</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Ministry of Agriculture &amp; Farmers Welfare, Government of India</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Programme Name</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B11" t="str">
         <v>AgriStack</v>
       </c>
-      <c r="C9" t="str">
-        <v/>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Programme Officer / POC</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v>Name of the nodal officer or point of contact.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Data Verified By</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v>Name of person who verified this data before import.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Data Verification Date</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v>Date of verification. Format: DD Month YYYY</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>API Base URL (future)</v>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v>When a real API is ready, enter the base URL here. e.g. https://api.agristack.gov.in</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixed the bug in CLI of preview
</commit_message>
<xml_diff>
--- a/scripts/AgriStack_Data_Template.xlsx
+++ b/scripts/AgriStack_Data_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/devansh/Projects/EY/dashboard/agristack-dashboard/scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB5994A7-1F55-C945-AADC-E6905DA5A677}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B66CBA-A031-5642-AFC1-8E8EC79C6AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUCTIONS" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1335" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1335" uniqueCount="349">
   <si>
     <t>AgriStack Dashboard — Data Entry Template  (v2)</t>
   </si>
@@ -978,9 +978,6 @@
     <t>Enrolled Farmers Last Updated</t>
   </si>
   <si>
-    <t>23 June 2026</t>
-  </si>
-  <si>
     <t>Date when the enrolled farmer count was last checked. Format: DD Month YYYY</t>
   </si>
   <si>
@@ -1068,7 +1065,28 @@
     <t>When a real API is ready, enter the base URL here. e.g. https://api.agristack.gov.in</t>
   </si>
   <si>
-    <t>UP,CG,MP,MH,AP,TG,RJ,TN</t>
+    <t>UP, MP, CG, MH, AP, TG, RJ, TN, GJ, AS</t>
+  </si>
+  <si>
+    <t>UP, CG, MH, GJ, AS</t>
+  </si>
+  <si>
+    <t>UP, MP, CG, MH, AP, TG, RJ, TN, GJ, AS, OD,KL, KA</t>
+  </si>
+  <si>
+    <t>UP, CG, PJ, GJ, AS, KL</t>
+  </si>
+  <si>
+    <t>MH</t>
+  </si>
+  <si>
+    <t>MP, CG, OD</t>
+  </si>
+  <si>
+    <t>UP, CG, AP, TG, RJ, TN, OD, GJ, AS, MN</t>
+  </si>
+  <si>
+    <t>24 June 2026</t>
   </si>
 </sst>
 </file>
@@ -1104,8 +1122,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2087,7 +2106,7 @@
         <v>3</v>
       </c>
       <c r="G2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H2" t="s">
         <v>121</v>
@@ -2125,7 +2144,7 @@
         <v>3</v>
       </c>
       <c r="G3" t="s">
-        <v>3</v>
+        <v>342</v>
       </c>
       <c r="H3" t="s">
         <v>124</v>
@@ -2163,7 +2182,7 @@
         <v>3</v>
       </c>
       <c r="G4" t="s">
-        <v>3</v>
+        <v>343</v>
       </c>
       <c r="H4" t="s">
         <v>127</v>
@@ -2201,7 +2220,7 @@
         <v>3</v>
       </c>
       <c r="G5" t="s">
-        <v>3</v>
+        <v>344</v>
       </c>
       <c r="H5" t="s">
         <v>130</v>
@@ -2239,7 +2258,7 @@
         <v>3</v>
       </c>
       <c r="G6" t="s">
-        <v>3</v>
+        <v>345</v>
       </c>
       <c r="H6" t="s">
         <v>3</v>
@@ -2277,7 +2296,7 @@
         <v>3</v>
       </c>
       <c r="G7" t="s">
-        <v>3</v>
+        <v>346</v>
       </c>
       <c r="H7" t="s">
         <v>133</v>
@@ -2505,7 +2524,7 @@
         <v>3</v>
       </c>
       <c r="G13" t="s">
-        <v>3</v>
+        <v>347</v>
       </c>
       <c r="H13" t="s">
         <v>144</v>
@@ -5034,7 +5053,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L1 A3:L79 A2:F2 H2:L2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L1 A8:L12 A2:F2 H2:L2 A3:F3 H3:L3 A4:F4 H4:L4 A5:F5 H5:L5 A6:F6 H6:L6 A7:F7 H7:L7 A14:L79 A13:F13 H13:L13" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6283,82 +6302,82 @@
       <c r="A3" t="s">
         <v>311</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C3" t="s">
         <v>312</v>
-      </c>
-      <c r="C3" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>313</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C4" t="s">
         <v>314</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>315</v>
+      </c>
+      <c r="B5" t="s">
         <v>316</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>317</v>
-      </c>
-      <c r="C5" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>318</v>
+      </c>
+      <c r="B6" t="s">
         <v>319</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>320</v>
-      </c>
-      <c r="C6" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>321</v>
+      </c>
+      <c r="B7" t="s">
         <v>322</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>323</v>
-      </c>
-      <c r="C7" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>324</v>
+      </c>
+      <c r="B8" t="s">
         <v>325</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>326</v>
-      </c>
-      <c r="C8" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>327</v>
+      </c>
+      <c r="B9" t="s">
         <v>328</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>329</v>
-      </c>
-      <c r="C9" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B10" t="s">
         <v>1</v>
@@ -6369,10 +6388,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>331</v>
+      </c>
+      <c r="B11" t="s">
         <v>332</v>
-      </c>
-      <c r="B11" t="s">
-        <v>333</v>
       </c>
       <c r="C11" t="s">
         <v>3</v>
@@ -6380,52 +6399,52 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>333</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
         <v>334</v>
-      </c>
-      <c r="B12" t="s">
-        <v>3</v>
-      </c>
-      <c r="C12" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>335</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
         <v>336</v>
-      </c>
-      <c r="B13" t="s">
-        <v>3</v>
-      </c>
-      <c r="C13" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>337</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
         <v>338</v>
-      </c>
-      <c r="B14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
+        <v>339</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
         <v>340</v>
-      </c>
-      <c r="B15" t="s">
-        <v>3</v>
-      </c>
-      <c r="C15" t="s">
-        <v>341</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C1 A3:C15 A2 C2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C1 A5:C15 A2 C2 A3 C3 A4 C4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data updated for the day
</commit_message>
<xml_diff>
--- a/scripts/AgriStack_Data_Template.xlsx
+++ b/scripts/AgriStack_Data_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/devansh/Projects/EY/dashboard/agristack-dashboard/scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B66CBA-A031-5642-AFC1-8E8EC79C6AA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C19C2580-AC33-0649-8CCA-E2DA9C689CDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19880" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1335" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1336" uniqueCount="351">
   <si>
     <t>AgriStack Dashboard — Data Entry Template  (v2)</t>
   </si>
@@ -1087,6 +1087,12 @@
   </si>
   <si>
     <t>24 June 2026</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>9.99 CR+</t>
   </si>
 </sst>
 </file>
@@ -5145,7 +5151,7 @@
         <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>349</v>
       </c>
       <c r="D3" t="s">
         <v>59</v>
@@ -6004,7 +6010,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J1 A3:J29 A2:C2 E2:J2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J1 A4:J29 A2:C2 E2:J2 A3:B3 D3:J3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6291,8 +6297,8 @@
       <c r="A2" t="s">
         <v>309</v>
       </c>
-      <c r="B2">
-        <v>99971794</v>
+      <c r="B2" t="s">
+        <v>350</v>
       </c>
       <c r="C2" t="s">
         <v>310</v>

</xml_diff>